<commit_message>
Add TG412 vapour MLP and aerosol LGB models with performance summary
</commit_message>
<xml_diff>
--- a/Final_model_save/ToxBAI_upload_needed/Inhalation_model/inhalation_models_summary.xlsx
+++ b/Final_model_save/ToxBAI_upload_needed/Inhalation_model/inhalation_models_summary.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="21" uniqueCount="18">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="27" uniqueCount="21">
   <si>
     <t>Model</t>
   </si>
@@ -55,6 +55,12 @@
     <t>TG413_vapour_RDKit_mlp_best</t>
   </si>
   <si>
+    <t>TG412_vapour_MACCS_mlp_best</t>
+  </si>
+  <si>
+    <t>TG412_aerosol_RDKit_lgb_best</t>
+  </si>
+  <si>
     <t>MACCS</t>
   </si>
   <si>
@@ -68,6 +74,9 @@
   </si>
   <si>
     <t>MLP</t>
+  </si>
+  <si>
+    <t>LGB</t>
   </si>
 </sst>
 </file>
@@ -425,7 +434,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:I5"/>
+  <dimension ref="A1:I7"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:9">
@@ -465,10 +474,10 @@
         <v>556</v>
       </c>
       <c r="C2" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="D2" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="E2">
         <v>0.3077</v>
@@ -494,10 +503,10 @@
         <v>455</v>
       </c>
       <c r="C3" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="D3" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="E3">
         <v>0.4103</v>
@@ -523,10 +532,10 @@
         <v>55</v>
       </c>
       <c r="C4" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="D4" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="E4">
         <v>0.4444</v>
@@ -552,10 +561,10 @@
         <v>239</v>
       </c>
       <c r="C5" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="D5" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="E5">
         <v>0.8354</v>
@@ -571,6 +580,64 @@
       </c>
       <c r="I5">
         <v>0.825</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9">
+      <c r="A6" t="s">
+        <v>13</v>
+      </c>
+      <c r="B6">
+        <v>210</v>
+      </c>
+      <c r="C6" t="s">
+        <v>15</v>
+      </c>
+      <c r="D6" t="s">
+        <v>19</v>
+      </c>
+      <c r="E6">
+        <v>0.6875</v>
+      </c>
+      <c r="F6">
+        <v>0.8355</v>
+      </c>
+      <c r="G6">
+        <v>0.7619</v>
+      </c>
+      <c r="H6">
+        <v>0.5789</v>
+      </c>
+      <c r="I6">
+        <v>0.8462</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9">
+      <c r="A7" t="s">
+        <v>14</v>
+      </c>
+      <c r="B7">
+        <v>77</v>
+      </c>
+      <c r="C7" t="s">
+        <v>17</v>
+      </c>
+      <c r="D7" t="s">
+        <v>20</v>
+      </c>
+      <c r="E7">
+        <v>0.4</v>
+      </c>
+      <c r="F7">
+        <v>0.6909</v>
+      </c>
+      <c r="G7">
+        <v>0.625</v>
+      </c>
+      <c r="H7">
+        <v>0.4</v>
+      </c>
+      <c r="I7">
+        <v>0.4</v>
       </c>
     </row>
   </sheetData>

</xml_diff>